<commit_message>
Execute test cases 1–3
</commit_message>
<xml_diff>
--- a/04-Test_Cases/01-Test_Cases.xlsx
+++ b/04-Test_Cases/01-Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\QADemo E-Commerce Application Manual Testing\QADemoE-CommerceApplicationManualTesting\04-Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E6BA104-B7FB-4E03-BECA-2569FD6A6217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40931C93-6505-46CE-97BA-5408B0720701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="539">
   <si>
     <t>Key</t>
   </si>
@@ -324,9 +324,6 @@
     <t>Valid registered customer credentials.</t>
   </si>
   <si>
-    <t>The system authenticates the customer and displays the appropriate authenticated page or account state.</t>
-  </si>
-  <si>
     <t>Positive</t>
   </si>
   <si>
@@ -345,12 +342,6 @@
 4. Submit the form.</t>
   </si>
   <si>
-    <t>Registered email; incorrect password.</t>
-  </si>
-  <si>
-    <t>Login is rejected, an appropriate error is displayed, and protected customer content is not accessible.</t>
-  </si>
-  <si>
     <t>Negative</t>
   </si>
   <si>
@@ -363,9 +354,6 @@
     <t>1. Enter an email/username not associated with a registered customer.
 2. Enter a password.
 3. Submit the form.</t>
-  </si>
-  <si>
-    <t>Unregistered email; arbitrary password.</t>
   </si>
   <si>
     <t>Login is rejected and the system does not create or authenticate an account.</t>
@@ -1762,12 +1750,54 @@
   <si>
     <t>Test Cases</t>
   </si>
+  <si>
+    <t>Username or Email: standard_user
+Password: standard123</t>
+  </si>
+  <si>
+    <t>The system should authenticate the user and display the status of the successfully authenticated account.</t>
+  </si>
+  <si>
+    <t>The system successfully displays the status of the authorized account.</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-1.jpg</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Username or Email: standard_user
+Password: tester124</t>
+  </si>
+  <si>
+    <t>The login should be rejected, an appropriate error message should be displayed and it must be ensured that protected customer content cannot be accessed.</t>
+  </si>
+  <si>
+    <t>The login is rejected, an appropriate error message is displayed and it is ensured that no one can access the customer's protected content.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-2.jpg</t>
+  </si>
+  <si>
+    <t>Username or Email: tester_user
+Password: standard123</t>
+  </si>
+  <si>
+    <t>Login should be rejected and the system should not create or authenticate an account.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-3.jpg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1787,6 +1817,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1813,7 +1849,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1830,6 +1866,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1837,39 +1876,7 @@
   </cellStyles>
   <dxfs count="21">
     <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1933,6 +1940,38 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1968,32 +2007,32 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC0972E8-E27C-45A1-BD68-74AC7D938AB0}" name="Table13" displayName="Table13" ref="A2:B9" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A2:B9" xr:uid="{AC0972E8-E27C-45A1-BD68-74AC7D938AB0}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{05A7F6E6-1E8F-4B9C-810B-C9396C6B5456}" name="Key" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{FFC49D79-8BCB-4241-9F71-306E1E028408}" name="Value" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{05A7F6E6-1E8F-4B9C-810B-C9396C6B5456}" name="Key" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{FFC49D79-8BCB-4241-9F71-306E1E028408}" name="Value" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}" name="Table2" displayName="Table2" ref="A13:O79" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}" name="Table2" displayName="Table2" ref="A13:O79" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A13:O79" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D243436B-E280-47D1-9048-A55E41BCCDA7}" name="Test Case ID" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{04E3F4CC-C517-4D34-AF59-7D35761EA7A2}" name="Test Case Title" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{B5CDD440-C8DB-4010-81FA-5ED0AE5FAC24}" name="Test Scenario ID" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{A2E98623-58F2-4087-AA4D-768C17D712B4}" name="Requirements ID" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{0948D040-2ED0-49D3-A3F7-D2DE67922DAC}" name="Module" dataDxfId="12"/>
-    <tableColumn id="20" xr3:uid="{4C1A7320-75FB-4DC9-B451-C7A962DC6823}" name="Test Type" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{7DAE9DF7-AED9-4464-B6F3-1D0B5E71B685}" name="Preconditions" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{6563B834-3510-45D1-A3BB-261DAA503DC2}" name="Test Steps" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{8A9D41F2-3075-43D5-9FCE-201D9AE235D8}" name="Test Data" dataDxfId="8"/>
-    <tableColumn id="19" xr3:uid="{C0B5DD96-4C37-470C-A90B-C0F6BAEE4561}" name="Expected Result" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{EBECA87A-F936-442B-813B-CB8A8FF2959A}" name="Actual Result" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{CE5B88B8-BB15-458C-8434-70F85E2E87E6}" name="Priority" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{C38F7409-03E4-49EE-B8AB-36C447EA718E}" name="Execution Status" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{3F9ED411-BFCC-43BC-9869-C0177649C0FB}" name="Defect ID" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{94FF1D6A-77E0-4094-9426-C2A41DEB43DF}" name="Remarks / Evidence" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D243436B-E280-47D1-9048-A55E41BCCDA7}" name="Test Case ID" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{04E3F4CC-C517-4D34-AF59-7D35761EA7A2}" name="Test Case Title" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B5CDD440-C8DB-4010-81FA-5ED0AE5FAC24}" name="Test Scenario ID" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{A2E98623-58F2-4087-AA4D-768C17D712B4}" name="Requirements ID" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{0948D040-2ED0-49D3-A3F7-D2DE67922DAC}" name="Module" dataDxfId="10"/>
+    <tableColumn id="20" xr3:uid="{4C1A7320-75FB-4DC9-B451-C7A962DC6823}" name="Test Type" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{7DAE9DF7-AED9-4464-B6F3-1D0B5E71B685}" name="Preconditions" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{6563B834-3510-45D1-A3BB-261DAA503DC2}" name="Test Steps" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{8A9D41F2-3075-43D5-9FCE-201D9AE235D8}" name="Test Data" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{C0B5DD96-4C37-470C-A90B-C0F6BAEE4561}" name="Expected Result" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{EBECA87A-F936-442B-813B-CB8A8FF2959A}" name="Actual Result" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{CE5B88B8-BB15-458C-8434-70F85E2E87E6}" name="Priority" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{C38F7409-03E4-49EE-B8AB-36C447EA718E}" name="Execution Status" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{3F9ED411-BFCC-43BC-9869-C0177649C0FB}" name="Defect ID" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{94FF1D6A-77E0-4094-9426-C2A41DEB43DF}" name="Remarks / Evidence" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2297,7 +2336,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>529</v>
+        <v>525</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -2326,7 +2365,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -2334,7 +2373,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -2342,10 +2381,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -2412,7 +2451,7 @@
         <v>94</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>95</v>
@@ -2421,28 +2460,36 @@
         <v>96</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>97</v>
+        <v>526</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="K14" s="3"/>
+        <v>527</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>528</v>
+      </c>
       <c r="L14" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="3"/>
-    </row>
-    <row r="15" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="O14" s="6" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>89</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>92</v>
@@ -2451,37 +2498,45 @@
         <v>94</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>95</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>104</v>
+        <v>532</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="K15" s="3"/>
+        <v>533</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>534</v>
+      </c>
       <c r="L15" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="3"/>
+        <v>99</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="16" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>92</v>
@@ -2490,37 +2545,45 @@
         <v>94</v>
       </c>
       <c r="F16" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>109</v>
-      </c>
       <c r="I16" s="3" t="s">
-        <v>110</v>
+        <v>536</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="K16" s="3"/>
+        <v>537</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="L16" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="3"/>
+        <v>99</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="17" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>92</v>
@@ -2529,37 +2592,37 @@
         <v>94</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="K17" s="3"/>
       <c r="L17" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
-      <c r="O17" s="3"/>
+      <c r="O17" s="2"/>
     </row>
     <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>92</v>
@@ -2568,37 +2631,37 @@
         <v>94</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>122</v>
-      </c>
       <c r="J18" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="K18" s="3"/>
       <c r="L18" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
-      <c r="O18" s="3"/>
+      <c r="O18" s="2"/>
     </row>
     <row r="19" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>85</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>92</v>
@@ -2607,37 +2670,37 @@
         <v>94</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="K19" s="3"/>
       <c r="L19" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
-      <c r="O19" s="3"/>
+      <c r="O19" s="2"/>
     </row>
     <row r="20" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>92</v>
@@ -2646,37 +2709,37 @@
         <v>94</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I20" s="3" t="s">
         <v>97</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="K20" s="3"/>
       <c r="L20" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
-      <c r="O20" s="3"/>
+      <c r="O20" s="2"/>
     </row>
     <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>92</v>
@@ -2685,37 +2748,37 @@
         <v>94</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="K21" s="3"/>
       <c r="L21" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="3"/>
+      <c r="O21" s="2"/>
     </row>
     <row r="22" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>92</v>
@@ -2724,1783 +2787,1783 @@
         <v>94</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="K22" s="3"/>
       <c r="L22" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
-      <c r="O22" s="3"/>
+      <c r="O22" s="2"/>
     </row>
     <row r="23" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I23" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="J23" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="J23" s="3" t="s">
-        <v>155</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
-      <c r="O23" s="3"/>
+      <c r="O23" s="2"/>
     </row>
     <row r="24" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="3"/>
+      <c r="O24" s="2"/>
     </row>
     <row r="25" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="I25" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E25" s="2" t="s">
+      <c r="J25" s="3" t="s">
         <v>165</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>169</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
-      <c r="O25" s="3"/>
+      <c r="O25" s="2"/>
     </row>
     <row r="26" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>170</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="3"/>
+      <c r="O26" s="2"/>
     </row>
     <row r="27" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>77</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I27" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E27" s="2" t="s">
+      <c r="J27" s="3" t="s">
         <v>178</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
-      <c r="O27" s="3"/>
+      <c r="O27" s="2"/>
     </row>
     <row r="28" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="J28" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
-      <c r="O28" s="3"/>
+      <c r="O28" s="2"/>
     </row>
     <row r="29" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="J29" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>194</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
-      <c r="O29" s="3"/>
+      <c r="O29" s="2"/>
     </row>
     <row r="30" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="J30" s="3" t="s">
         <v>195</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
-      <c r="O30" s="3"/>
+      <c r="O30" s="2"/>
     </row>
     <row r="31" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="I31" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="J31" s="3" t="s">
         <v>203</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>207</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
-      <c r="O31" s="3"/>
+      <c r="O31" s="2"/>
     </row>
     <row r="32" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>213</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
-      <c r="O32" s="3"/>
+      <c r="O32" s="2"/>
     </row>
     <row r="33" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="J33" s="3" t="s">
         <v>215</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>219</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
-      <c r="O33" s="3"/>
+      <c r="O33" s="2"/>
     </row>
     <row r="34" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="J34" s="3" t="s">
         <v>221</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>225</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
-      <c r="O34" s="3"/>
+      <c r="O34" s="2"/>
     </row>
     <row r="35" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>69</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="J35" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>231</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
-      <c r="O35" s="3"/>
+      <c r="O35" s="2"/>
     </row>
     <row r="36" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F36" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>236</v>
-      </c>
       <c r="G36" s="3" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
-      <c r="O36" s="3"/>
+      <c r="O36" s="2"/>
     </row>
     <row r="37" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>242</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
-      <c r="O37" s="3"/>
+      <c r="O37" s="2"/>
     </row>
     <row r="38" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="J38" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>247</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
-      <c r="O38" s="3"/>
+      <c r="O38" s="2"/>
     </row>
     <row r="39" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="J39" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
-      <c r="O39" s="3"/>
+      <c r="O39" s="2"/>
     </row>
     <row r="40" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>64</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="I40" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E40" s="2" t="s">
+      <c r="J40" s="3" t="s">
         <v>257</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>261</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
-      <c r="O40" s="3"/>
+      <c r="O40" s="2"/>
     </row>
     <row r="41" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="J41" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>267</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
-      <c r="O41" s="3"/>
+      <c r="O41" s="2"/>
     </row>
     <row r="42" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="J42" s="3" t="s">
         <v>269</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
-      <c r="O42" s="3"/>
+      <c r="O42" s="2"/>
     </row>
     <row r="43" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="J43" s="3" t="s">
         <v>275</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="J43" s="3" t="s">
-        <v>279</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
-      <c r="O43" s="3"/>
+      <c r="O43" s="2"/>
     </row>
     <row r="44" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="J44" s="3" t="s">
         <v>281</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="J44" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="K44" s="3"/>
       <c r="L44" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
-      <c r="O44" s="3"/>
+      <c r="O44" s="2"/>
     </row>
     <row r="45" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="I45" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="E45" s="2" t="s">
+      <c r="J45" s="3" t="s">
         <v>289</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>290</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="J45" s="3" t="s">
-        <v>293</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
-      <c r="O45" s="3"/>
+      <c r="O45" s="2"/>
     </row>
     <row r="46" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F46" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="G46" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="J46" s="3" t="s">
         <v>295</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="J46" s="3" t="s">
-        <v>299</v>
       </c>
       <c r="K46" s="3"/>
       <c r="L46" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
-      <c r="O46" s="3"/>
+      <c r="O46" s="2"/>
     </row>
     <row r="47" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="J47" s="3" t="s">
         <v>302</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="I47" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="J47" s="3" t="s">
-        <v>306</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
-      <c r="O47" s="3"/>
+      <c r="O47" s="2"/>
     </row>
     <row r="48" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>56</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
-      <c r="O48" s="3"/>
+      <c r="O48" s="2"/>
     </row>
     <row r="49" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="K49" s="3"/>
       <c r="L49" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2"/>
-      <c r="O49" s="3"/>
+      <c r="O49" s="2"/>
     </row>
     <row r="50" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="I50" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E50" s="2" t="s">
+      <c r="J50" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="J50" s="3" t="s">
-        <v>323</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M50" s="2"/>
       <c r="N50" s="2"/>
-      <c r="O50" s="3"/>
+      <c r="O50" s="2"/>
     </row>
     <row r="51" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="J51" s="3" t="s">
         <v>326</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>325</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G51" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="H51" s="3" t="s">
-        <v>328</v>
-      </c>
-      <c r="I51" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="J51" s="3" t="s">
-        <v>330</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M51" s="2"/>
       <c r="N51" s="2"/>
-      <c r="O51" s="3"/>
+      <c r="O51" s="2"/>
     </row>
     <row r="52" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="J52" s="3" t="s">
         <v>331</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="J52" s="3" t="s">
-        <v>335</v>
       </c>
       <c r="K52" s="3"/>
       <c r="L52" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
-      <c r="O52" s="3"/>
+      <c r="O52" s="2"/>
     </row>
     <row r="53" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="I53" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="C53" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="E53" s="2" t="s">
+      <c r="J53" s="3" t="s">
         <v>340</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="I53" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="J53" s="3" t="s">
-        <v>344</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M53" s="2"/>
       <c r="N53" s="2"/>
-      <c r="O53" s="3"/>
+      <c r="O53" s="2"/>
     </row>
     <row r="54" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="J54" s="3" t="s">
         <v>346</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>345</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="J54" s="3" t="s">
-        <v>350</v>
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M54" s="2"/>
       <c r="N54" s="2"/>
-      <c r="O54" s="3"/>
+      <c r="O54" s="2"/>
     </row>
     <row r="55" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="I55" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E55" s="2" t="s">
+      <c r="J55" s="3" t="s">
         <v>354</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="I55" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="J55" s="3" t="s">
-        <v>358</v>
       </c>
       <c r="K55" s="3"/>
       <c r="L55" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
-      <c r="O55" s="3"/>
+      <c r="O55" s="2"/>
     </row>
     <row r="56" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="J56" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>362</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>363</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M56" s="2"/>
       <c r="N56" s="2"/>
-      <c r="O56" s="3"/>
+      <c r="O56" s="2"/>
     </row>
     <row r="57" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="J57" s="3" t="s">
         <v>365</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G57" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="H57" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>368</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>369</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M57" s="2"/>
       <c r="N57" s="2"/>
-      <c r="O57" s="3"/>
+      <c r="O57" s="2"/>
     </row>
     <row r="58" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B58" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>369</v>
+      </c>
+      <c r="J58" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="J58" s="3" t="s">
-        <v>374</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
-      <c r="O58" s="3"/>
+      <c r="O58" s="2"/>
     </row>
     <row r="59" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="J59" s="3" t="s">
         <v>376</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="G59" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="H59" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="J59" s="3" t="s">
-        <v>380</v>
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
-      <c r="O59" s="3"/>
+      <c r="O59" s="2"/>
     </row>
     <row r="60" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="J60" s="3" t="s">
         <v>381</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>384</v>
-      </c>
-      <c r="J60" s="3" t="s">
-        <v>385</v>
       </c>
       <c r="K60" s="3"/>
       <c r="L60" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M60" s="2"/>
       <c r="N60" s="2"/>
-      <c r="O60" s="3"/>
+      <c r="O60" s="2"/>
     </row>
     <row r="61" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="J61" s="3" t="s">
         <v>387</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="H61" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="I61" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="J61" s="3" t="s">
-        <v>391</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
-      <c r="O61" s="3"/>
+      <c r="O61" s="2"/>
     </row>
     <row r="62" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="C62" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="J62" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="J62" s="3" t="s">
-        <v>396</v>
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
-      <c r="O62" s="3"/>
+      <c r="O62" s="2"/>
     </row>
     <row r="63" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="J63" s="3" t="s">
         <v>397</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>402</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="J63" s="3" t="s">
-        <v>401</v>
       </c>
       <c r="K63" s="3"/>
       <c r="L63" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M63" s="2"/>
       <c r="N63" s="2"/>
-      <c r="O63" s="3"/>
+      <c r="O63" s="2"/>
     </row>
     <row r="64" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="I64" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="E64" s="2" t="s">
+      <c r="J64" s="3" t="s">
         <v>406</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="G64" s="3" t="s">
-        <v>407</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="I64" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="J64" s="3" t="s">
-        <v>410</v>
       </c>
       <c r="K64" s="3"/>
       <c r="L64" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M64" s="2"/>
       <c r="N64" s="2"/>
-      <c r="O64" s="3"/>
+      <c r="O64" s="2"/>
     </row>
     <row r="65" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="C65" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="G65" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>407</v>
-      </c>
       <c r="H65" s="3" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="I65" s="3" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="J65" s="3" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="K65" s="3"/>
       <c r="L65" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
-      <c r="O65" s="3"/>
+      <c r="O65" s="2"/>
     </row>
     <row r="66" spans="1:15" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B66" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="I66" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="E66" s="2" t="s">
+      <c r="J66" s="3" t="s">
         <v>418</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>421</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>422</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
-      <c r="O66" s="3"/>
+      <c r="O66" s="2"/>
     </row>
     <row r="67" spans="1:15" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="I67" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="C67" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="E67" s="2" t="s">
+      <c r="J67" s="3" t="s">
         <v>427</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>428</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>430</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>431</v>
       </c>
       <c r="K67" s="3"/>
       <c r="L67" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
-      <c r="O67" s="3" t="s">
-        <v>432</v>
+      <c r="O67" s="2" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4508,272 +4571,274 @@
         <v>36</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="J68" s="3" t="s">
         <v>435</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="H68" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="I68" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="J68" s="3" t="s">
-        <v>439</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M68" s="2"/>
       <c r="N68" s="2"/>
-      <c r="O68" s="3"/>
+      <c r="O68" s="2"/>
     </row>
     <row r="69" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B69" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="J69" s="3" t="s">
         <v>440</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>441</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>442</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>443</v>
-      </c>
-      <c r="J69" s="3" t="s">
-        <v>444</v>
       </c>
       <c r="K69" s="3"/>
       <c r="L69" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M69" s="2"/>
       <c r="N69" s="2"/>
-      <c r="O69" s="3"/>
+      <c r="O69" s="2"/>
     </row>
     <row r="70" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B70" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="I70" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="E70" s="2" t="s">
+      <c r="J70" s="3" t="s">
         <v>448</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>449</v>
-      </c>
-      <c r="H70" s="3" t="s">
-        <v>450</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>451</v>
-      </c>
-      <c r="J70" s="3" t="s">
-        <v>452</v>
       </c>
       <c r="K70" s="3"/>
       <c r="L70" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M70" s="2"/>
       <c r="N70" s="2"/>
-      <c r="O70" s="3"/>
+      <c r="O70" s="2"/>
     </row>
     <row r="71" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="I71" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="C71" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="E71" s="2" t="s">
+      <c r="J71" s="3" t="s">
         <v>457</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>458</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="J71" s="3" t="s">
-        <v>461</v>
       </c>
       <c r="K71" s="3"/>
       <c r="L71" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M71" s="2"/>
       <c r="N71" s="2"/>
-      <c r="O71" s="3"/>
+      <c r="O71" s="2"/>
     </row>
     <row r="72" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B72" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="J72" s="3" t="s">
         <v>464</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>465</v>
-      </c>
-      <c r="H72" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="I72" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="J72" s="3" t="s">
-        <v>468</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M72" s="2"/>
       <c r="N72" s="2"/>
-      <c r="O72" s="3"/>
+      <c r="O72" s="2"/>
     </row>
     <row r="73" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="I73" s="3" t="s">
         <v>472</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="E73" s="2" t="s">
+      <c r="J73" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>474</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="J73" s="3" t="s">
-        <v>477</v>
       </c>
       <c r="K73" s="3"/>
       <c r="L73" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M73" s="2"/>
       <c r="N73" s="2"/>
-      <c r="O73" s="3"/>
+      <c r="O73" s="2"/>
     </row>
     <row r="74" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="I74" s="3" t="s">
         <v>479</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2" t="s">
+      <c r="J74" s="3" t="s">
         <v>480</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="H74" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="I74" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="J74" s="3" t="s">
-        <v>484</v>
       </c>
       <c r="K74" s="3"/>
       <c r="L74" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
-      <c r="O74" s="3" t="s">
-        <v>486</v>
+      <c r="O74" s="2" t="s">
+        <v>482</v>
       </c>
     </row>
     <row r="75" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
@@ -4781,38 +4846,40 @@
         <v>29</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="J75" s="3" t="s">
         <v>488</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>489</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>490</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="J75" s="3" t="s">
-        <v>492</v>
       </c>
       <c r="K75" s="3"/>
       <c r="L75" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M75" s="2"/>
       <c r="N75" s="2"/>
-      <c r="O75" s="3" t="s">
-        <v>494</v>
+      <c r="O75" s="2" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4820,38 +4887,40 @@
         <v>28</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="I76" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2" t="s">
+      <c r="J76" s="3" t="s">
         <v>497</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>498</v>
-      </c>
-      <c r="H76" s="3" t="s">
-        <v>499</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>500</v>
-      </c>
-      <c r="J76" s="3" t="s">
-        <v>501</v>
       </c>
       <c r="K76" s="3"/>
       <c r="L76" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M76" s="2"/>
       <c r="N76" s="2"/>
-      <c r="O76" s="3" t="s">
-        <v>503</v>
+      <c r="O76" s="2" t="s">
+        <v>499</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4859,124 +4928,130 @@
         <v>27</v>
       </c>
       <c r="B77" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="J77" s="3" t="s">
         <v>505</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="F77" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>506</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>508</v>
-      </c>
-      <c r="J77" s="3" t="s">
-        <v>509</v>
       </c>
       <c r="K77" s="3"/>
       <c r="L77" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M77" s="2"/>
       <c r="N77" s="2"/>
-      <c r="O77" s="3"/>
+      <c r="O77" s="2"/>
     </row>
     <row r="78" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>511</v>
+      </c>
+      <c r="I78" s="3" t="s">
         <v>512</v>
       </c>
-      <c r="C78" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="E78" s="2" t="s">
+      <c r="J78" s="3" t="s">
         <v>513</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>514</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>515</v>
-      </c>
-      <c r="I78" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="J78" s="3" t="s">
-        <v>517</v>
       </c>
       <c r="K78" s="3"/>
       <c r="L78" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="M78" s="2"/>
       <c r="N78" s="2"/>
-      <c r="O78" s="3"/>
+      <c r="O78" s="2"/>
     </row>
     <row r="79" spans="1:15" ht="216" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>517</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="I79" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="E79" s="2" t="s">
+      <c r="J79" s="3" t="s">
         <v>520</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="G79" s="3" t="s">
-        <v>521</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>522</v>
-      </c>
-      <c r="I79" s="3" t="s">
-        <v>523</v>
-      </c>
-      <c r="J79" s="3" t="s">
-        <v>524</v>
       </c>
       <c r="K79" s="3"/>
       <c r="L79" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
-      <c r="O79" s="3"/>
+      <c r="O79" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1" xr:uid="{A9C43836-539D-4081-8B35-8FEAFF66F00B}"/>
+    <hyperlink ref="O14" r:id="rId2" xr:uid="{6E2448A7-3E3A-4EC7-9A26-9D691343DC32}"/>
+    <hyperlink ref="O15" r:id="rId3" xr:uid="{627F729D-B612-4F71-80F2-BB40F6B19489}"/>
+    <hyperlink ref="O16" r:id="rId4" xr:uid="{939D41DA-AB41-4833-AC20-2A2CD4EE4F47}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Execute test cases 4-9
</commit_message>
<xml_diff>
--- a/04-Test_Cases/01-Test_Cases.xlsx
+++ b/04-Test_Cases/01-Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\QADemo E-Commerce Application Manual Testing\QADemoE-CommerceApplicationManualTesting\04-Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40931C93-6505-46CE-97BA-5408B0720701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0198C589-D620-4D68-9915-48C975877E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="550">
   <si>
     <t>Key</t>
   </si>
@@ -321,9 +321,6 @@
 4. Submit the form.</t>
   </si>
   <si>
-    <t>Valid registered customer credentials.</t>
-  </si>
-  <si>
     <t>Positive</t>
   </si>
   <si>
@@ -372,12 +369,6 @@
 2. Submit the form.</t>
   </si>
   <si>
-    <t>Both fields empty.</t>
-  </si>
-  <si>
-    <t>The system prevents login and identifies the required fields with appropriate validation feedback.</t>
-  </si>
-  <si>
     <t>Negative / Validation</t>
   </si>
   <si>
@@ -392,12 +383,6 @@
 3. Submit the form.</t>
   </si>
   <si>
-    <t>Registered email; blank password.</t>
-  </si>
-  <si>
-    <t>The system prevents login and provides validation feedback for the missing password.</t>
-  </si>
-  <si>
     <t>TS-004</t>
   </si>
   <si>
@@ -407,9 +392,6 @@
     <t>1. Click the password field.
 2. Type a password.
 3. Observe how the characters are displayed.</t>
-  </si>
-  <si>
-    <t>Password: QaDemo@123</t>
   </si>
   <si>
     <t>Password characters are obscured by default and are not displayed as readable plain text.</t>
@@ -436,9 +418,6 @@
 4. Observe the destination page and authentication state.</t>
   </si>
   <si>
-    <t>The customer is redirected to the appropriate page defined by the application and remains authenticated.</t>
-  </si>
-  <si>
     <t>TS-006</t>
   </si>
   <si>
@@ -453,9 +432,6 @@
   </si>
   <si>
     <t>Authenticated customer session.</t>
-  </si>
-  <si>
-    <t>The session is terminated and the customer is returned to the appropriate unauthenticated page.</t>
   </si>
   <si>
     <t>Prevent access to protected page after logout</t>
@@ -1791,6 +1767,65 @@
   </si>
   <si>
     <t>..\Evidence\TC-3.jpg</t>
+  </si>
+  <si>
+    <t>Both fields empty</t>
+  </si>
+  <si>
+    <t>The system's login process should be restricted and the required fields should be identified through appropriate validation feedback.</t>
+  </si>
+  <si>
+    <t>The system's login process is restricted, and the required fields are identified through appropriate validation feedback.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-4.jpg</t>
+  </si>
+  <si>
+    <t>Username or Email: standard_user
+Password:</t>
+  </si>
+  <si>
+    <t>The system should prevent login and provide feedback regarding the absence of a password.</t>
+  </si>
+  <si>
+    <t>The system prevents login and provides feedback regarding the absence of a password.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-5.jpg</t>
+  </si>
+  <si>
+    <t>Password characters should be hidden by default and should not be displayed as readable plain text.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-6.jpg</t>
+  </si>
+  <si>
+    <t>Username or Email: standard_user
+Password: standard124</t>
+  </si>
+  <si>
+    <t>The user should be redirected to an appropriate page determined by the application and must remain in an authenticated state.</t>
+  </si>
+  <si>
+    <t>The user is redirected to an appropriate page determined by the application and  remains in an authenticated state.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-7.jpg</t>
+  </si>
+  <si>
+    <t>The session should be terminated and the customer should be redirected to the appropriate unauthenticated page.</t>
+  </si>
+  <si>
+    <t>The session is terminated and the customer is redirected to the appropriate unauthenticated page.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-8.jpg</t>
+  </si>
+  <si>
+    <t>Protected information should not accessible using the terminated session; the customer should be redirected or asked to log in.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-9.jpg</t>
   </si>
 </sst>
 </file>
@@ -2336,7 +2371,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -2365,7 +2400,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -2373,7 +2408,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -2381,10 +2416,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -2451,7 +2486,7 @@
         <v>94</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>95</v>
@@ -2460,25 +2495,25 @@
         <v>96</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2486,10 +2521,10 @@
         <v>89</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>92</v>
@@ -2498,34 +2533,34 @@
         <v>94</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>95</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>532</v>
+        <v>524</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2533,10 +2568,10 @@
         <v>88</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>92</v>
@@ -2545,45 +2580,45 @@
         <v>94</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
+        <v>528</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>529</v>
+      </c>
+      <c r="K16" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="I16" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>107</v>
-      </c>
       <c r="L16" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>87</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>92</v>
@@ -2592,37 +2627,45 @@
         <v>94</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="H17" s="3" t="s">
-        <v>111</v>
-      </c>
       <c r="I17" s="3" t="s">
+        <v>531</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>533</v>
+      </c>
+      <c r="L17" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="J17" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K17" s="3"/>
-      <c r="L17" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+      <c r="M17" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>534</v>
+      </c>
     </row>
     <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>86</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>92</v>
@@ -2631,37 +2674,45 @@
         <v>94</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="I18" s="3" t="s">
-        <v>118</v>
+        <v>535</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="K18" s="3"/>
+        <v>536</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>537</v>
+      </c>
       <c r="L18" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="19" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>85</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>92</v>
@@ -2670,37 +2721,45 @@
         <v>94</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>123</v>
+        <v>518</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="K19" s="3"/>
+        <v>539</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>118</v>
+      </c>
       <c r="L19" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
+        <v>120</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>540</v>
+      </c>
     </row>
     <row r="20" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>84</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>92</v>
@@ -2709,37 +2768,45 @@
         <v>94</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>97</v>
+        <v>541</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="K20" s="3"/>
+        <v>542</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>543</v>
+      </c>
       <c r="L20" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>83</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>92</v>
@@ -2748,37 +2815,45 @@
         <v>94</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="K21" s="3"/>
+        <v>545</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>546</v>
+      </c>
       <c r="L21" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>547</v>
+      </c>
     </row>
     <row r="22" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>92</v>
@@ -2787,62 +2862,70 @@
         <v>94</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="K22" s="3"/>
+        <v>548</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="L22" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
+        <v>98</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="O22" s="6" t="s">
+        <v>549</v>
+      </c>
     </row>
     <row r="23" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="K23" s="3"/>
       <c r="L23" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
@@ -2853,35 +2936,35 @@
         <v>80</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="H24" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I24" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>155</v>
-      </c>
       <c r="J24" s="3" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="K24" s="3"/>
       <c r="L24" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
@@ -2892,35 +2975,35 @@
         <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="K25" s="3"/>
       <c r="L25" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
@@ -2931,35 +3014,35 @@
         <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G26" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="H26" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="I26" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>169</v>
-      </c>
       <c r="J26" s="3" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="K26" s="3"/>
       <c r="L26" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
@@ -2970,35 +3053,35 @@
         <v>77</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
@@ -3009,35 +3092,35 @@
         <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G28" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="H28" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="I28" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>182</v>
-      </c>
       <c r="J28" s="3" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
@@ -3048,35 +3131,35 @@
         <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -3087,35 +3170,35 @@
         <v>74</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="H30" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>193</v>
-      </c>
       <c r="I30" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
@@ -3126,35 +3209,35 @@
         <v>73</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -3165,35 +3248,35 @@
         <v>72</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E32" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="G32" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>207</v>
-      </c>
       <c r="I32" s="3" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
@@ -3204,35 +3287,35 @@
         <v>71</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
@@ -3243,35 +3326,35 @@
         <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
@@ -3282,35 +3365,35 @@
         <v>69</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
@@ -3321,35 +3404,35 @@
         <v>68</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="I36" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="J36" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
@@ -3360,35 +3443,35 @@
         <v>67</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
@@ -3399,35 +3482,35 @@
         <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="H38" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>241</v>
-      </c>
       <c r="I38" s="3" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
@@ -3438,35 +3521,35 @@
         <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
@@ -3477,35 +3560,35 @@
         <v>64</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>258</v>
-      </c>
       <c r="G40" s="3" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
@@ -3516,35 +3599,35 @@
         <v>63</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E41" s="2" t="s">
+      <c r="G41" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>261</v>
-      </c>
       <c r="I41" s="3" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
@@ -3555,35 +3638,35 @@
         <v>62</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F42" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>266</v>
-      </c>
       <c r="H42" s="3" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
@@ -3594,35 +3677,35 @@
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
@@ -3633,35 +3716,35 @@
         <v>60</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="G44" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>278</v>
-      </c>
       <c r="H44" s="3" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="K44" s="3"/>
       <c r="L44" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M44" s="2"/>
       <c r="N44" s="2"/>
@@ -3672,35 +3755,35 @@
         <v>59</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>290</v>
-      </c>
       <c r="G45" s="3" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
@@ -3711,35 +3794,35 @@
         <v>58</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="E46" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="G46" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="F46" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>293</v>
-      </c>
       <c r="H46" s="3" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="K46" s="3"/>
       <c r="L46" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
@@ -3750,35 +3833,35 @@
         <v>57</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M47" s="2"/>
       <c r="N47" s="2"/>
@@ -3789,35 +3872,35 @@
         <v>56</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="H48" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G48" s="3" t="s">
+      <c r="I48" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="J48" s="3" t="s">
         <v>299</v>
-      </c>
-      <c r="H48" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>307</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
@@ -3828,35 +3911,35 @@
         <v>55</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="K49" s="3"/>
       <c r="L49" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M49" s="2"/>
       <c r="N49" s="2"/>
@@ -3867,35 +3950,35 @@
         <v>54</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F50" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="G50" s="3" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M50" s="2"/>
       <c r="N50" s="2"/>
@@ -3906,35 +3989,35 @@
         <v>53</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="E51" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G51" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G51" s="3" t="s">
-        <v>323</v>
-      </c>
       <c r="H51" s="3" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M51" s="2"/>
       <c r="N51" s="2"/>
@@ -3945,35 +4028,35 @@
         <v>52</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="K52" s="3"/>
       <c r="L52" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
@@ -3984,35 +4067,35 @@
         <v>51</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M53" s="2"/>
       <c r="N53" s="2"/>
@@ -4023,35 +4106,35 @@
         <v>50</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="E54" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="H54" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="F54" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>344</v>
-      </c>
       <c r="I54" s="3" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M54" s="2"/>
       <c r="N54" s="2"/>
@@ -4062,35 +4145,35 @@
         <v>49</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="K55" s="3"/>
       <c r="L55" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
@@ -4101,35 +4184,35 @@
         <v>48</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="D56" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G56" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="H56" s="3" t="s">
+        <v>349</v>
+      </c>
+      <c r="I56" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>358</v>
-      </c>
       <c r="J56" s="3" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M56" s="2"/>
       <c r="N56" s="2"/>
@@ -4140,35 +4223,35 @@
         <v>47</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M57" s="2"/>
       <c r="N57" s="2"/>
@@ -4179,35 +4262,35 @@
         <v>46</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>366</v>
+        <v>358</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="H58" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>368</v>
-      </c>
       <c r="I58" s="3" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
@@ -4218,35 +4301,35 @@
         <v>45</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>372</v>
+        <v>364</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>371</v>
+        <v>363</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
@@ -4257,35 +4340,35 @@
         <v>44</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="H60" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>332</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>379</v>
-      </c>
       <c r="I60" s="3" t="s">
-        <v>380</v>
+        <v>372</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>381</v>
+        <v>373</v>
       </c>
       <c r="K60" s="3"/>
       <c r="L60" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M60" s="2"/>
       <c r="N60" s="2"/>
@@ -4296,35 +4379,35 @@
         <v>43</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>383</v>
+        <v>375</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>382</v>
+        <v>374</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>384</v>
+        <v>376</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>385</v>
+        <v>377</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
@@ -4335,35 +4418,35 @@
         <v>42</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>389</v>
+        <v>381</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>388</v>
+        <v>380</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>390</v>
+        <v>382</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>391</v>
+        <v>383</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
@@ -4374,35 +4457,35 @@
         <v>41</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>386</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="I63" s="3" t="s">
         <v>388</v>
       </c>
-      <c r="D63" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>396</v>
-      </c>
       <c r="J63" s="3" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="K63" s="3"/>
       <c r="L63" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M63" s="2"/>
       <c r="N63" s="2"/>
@@ -4413,35 +4496,35 @@
         <v>40</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>401</v>
+        <v>393</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>402</v>
+        <v>394</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>403</v>
+        <v>395</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>404</v>
+        <v>396</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="K64" s="3"/>
       <c r="L64" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M64" s="2"/>
       <c r="N64" s="2"/>
@@ -4452,35 +4535,35 @@
         <v>39</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>407</v>
+        <v>399</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>399</v>
+        <v>391</v>
       </c>
       <c r="D65" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="H65" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="I65" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="J65" s="3" t="s">
         <v>402</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>403</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="J65" s="3" t="s">
-        <v>410</v>
       </c>
       <c r="K65" s="3"/>
       <c r="L65" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
@@ -4491,35 +4574,35 @@
         <v>38</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F66" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>419</v>
-      </c>
       <c r="G66" s="3" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="I66" s="3" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
@@ -4530,40 +4613,40 @@
         <v>37</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>420</v>
+        <v>412</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="I67" s="3" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="K67" s="3"/>
       <c r="L67" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4571,35 +4654,35 @@
         <v>36</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M68" s="2"/>
       <c r="N68" s="2"/>
@@ -4610,35 +4693,35 @@
         <v>35</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>436</v>
+        <v>428</v>
       </c>
       <c r="C69" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G69" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="D69" s="2" t="s">
+      <c r="H69" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="E69" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>437</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>438</v>
-      </c>
       <c r="I69" s="3" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>440</v>
+        <v>432</v>
       </c>
       <c r="K69" s="3"/>
       <c r="L69" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M69" s="2"/>
       <c r="N69" s="2"/>
@@ -4649,35 +4732,35 @@
         <v>34</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="F70" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>449</v>
-      </c>
       <c r="G70" s="3" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="J70" s="3" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="K70" s="3"/>
       <c r="L70" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M70" s="2"/>
       <c r="N70" s="2"/>
@@ -4688,35 +4771,35 @@
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="F71" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="D71" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>458</v>
-      </c>
       <c r="G71" s="3" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="K71" s="3"/>
       <c r="L71" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M71" s="2"/>
       <c r="N71" s="2"/>
@@ -4727,35 +4810,35 @@
         <v>32</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>451</v>
+        <v>443</v>
       </c>
       <c r="E72" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="G72" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="F72" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>461</v>
-      </c>
       <c r="H72" s="3" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="M72" s="2"/>
       <c r="N72" s="2"/>
@@ -4766,35 +4849,35 @@
         <v>31</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>467</v>
+        <v>459</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>471</v>
+        <v>463</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="K73" s="3"/>
       <c r="L73" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M73" s="2"/>
       <c r="N73" s="2"/>
@@ -4805,40 +4888,40 @@
         <v>30</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>475</v>
+        <v>467</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>479</v>
+        <v>471</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="K74" s="3"/>
       <c r="L74" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
     </row>
     <row r="75" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
@@ -4846,40 +4929,40 @@
         <v>29</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="J75" s="3" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="K75" s="3"/>
       <c r="L75" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M75" s="2"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4887,40 +4970,40 @@
         <v>28</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>491</v>
+        <v>483</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>495</v>
+        <v>487</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="J76" s="3" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="K76" s="3"/>
       <c r="L76" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M76" s="2"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2" t="s">
-        <v>499</v>
+        <v>491</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4928,35 +5011,35 @@
         <v>27</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="J77" s="3" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="K77" s="3"/>
       <c r="L77" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M77" s="2"/>
       <c r="N77" s="2"/>
@@ -4967,35 +5050,35 @@
         <v>26</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>511</v>
+        <v>503</v>
       </c>
       <c r="I78" s="3" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="K78" s="3"/>
       <c r="L78" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="M78" s="2"/>
       <c r="N78" s="2"/>
@@ -5006,35 +5089,35 @@
         <v>25</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>515</v>
+        <v>507</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>507</v>
+        <v>499</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="K79" s="3"/>
       <c r="L79" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M79" s="2"/>
       <c r="N79" s="2"/>
@@ -5047,11 +5130,17 @@
     <hyperlink ref="O14" r:id="rId2" xr:uid="{6E2448A7-3E3A-4EC7-9A26-9D691343DC32}"/>
     <hyperlink ref="O15" r:id="rId3" xr:uid="{627F729D-B612-4F71-80F2-BB40F6B19489}"/>
     <hyperlink ref="O16" r:id="rId4" xr:uid="{939D41DA-AB41-4833-AC20-2A2CD4EE4F47}"/>
+    <hyperlink ref="O17" r:id="rId5" xr:uid="{E3D7EFC8-DC8F-4EF9-9C86-F8ADEDB90E8B}"/>
+    <hyperlink ref="O18" r:id="rId6" xr:uid="{E3FC0247-8964-4098-BAB0-3D9ACDFFEB2A}"/>
+    <hyperlink ref="O19" r:id="rId7" xr:uid="{E21557BB-CD23-4E7E-B329-472799E0A129}"/>
+    <hyperlink ref="O20" r:id="rId8" xr:uid="{F5787B2D-5828-4623-8A64-5D9CFF9E641B}"/>
+    <hyperlink ref="O21" r:id="rId9" xr:uid="{D4758FBB-2393-4158-82C5-88B1B57F3D54}"/>
+    <hyperlink ref="O22" r:id="rId10" xr:uid="{046CBEDE-BA76-4650-974F-62FAF5F2D2F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId5"/>
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Execute test cases 10-13
</commit_message>
<xml_diff>
--- a/04-Test_Cases/01-Test_Cases.xlsx
+++ b/04-Test_Cases/01-Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\QADemo E-Commerce Application Manual Testing\QADemoE-CommerceApplicationManualTesting\04-Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0198C589-D620-4D68-9915-48C975877E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71B03D3-63A4-45DC-A51D-7BADAD0CC11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="560">
   <si>
     <t>Key</t>
   </si>
@@ -476,9 +476,6 @@
     <t>Available products in the catalogue.</t>
   </si>
   <si>
-    <t>Available products are displayed with the relevant basic information, such as product name and price where provided by the UI.</t>
-  </si>
-  <si>
     <t>Display multiple available products</t>
   </si>
   <si>
@@ -523,9 +520,6 @@
     <t>Keyword: a known product name or distinctive term.</t>
   </si>
   <si>
-    <t>Search results include relevant matching products and allow the customer to identify the intended product.</t>
-  </si>
-  <si>
     <t>Show no-results feedback for an unmatched keyword</t>
   </si>
   <si>
@@ -538,9 +532,6 @@
   </si>
   <si>
     <t>Keyword: QZQ-NO-MATCH-98765</t>
-  </si>
-  <si>
-    <t>The system clearly indicates that no matching products were found; unrelated products are not presented as matches.</t>
   </si>
   <si>
     <t>TS-009</t>
@@ -1826,6 +1817,45 @@
   </si>
   <si>
     <t>..\Evidence\TC-9.jpg</t>
+  </si>
+  <si>
+    <t>Available products should be displayed with the relevant basic information.</t>
+  </si>
+  <si>
+    <t>Available products are displayed with the relevant basic information.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-10.jpg</t>
+  </si>
+  <si>
+    <t>The list should display the available products and their relevant information, ensuring that there are no unintended omissions or duplicate entries.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-11.jpg</t>
+  </si>
+  <si>
+    <t>Search results should include relevant and suitable products, so that the customer can identify the product they are looking for.</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>There is no search bar or search field for searching products.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-12.jpg</t>
+  </si>
+  <si>
+    <t>BUG-001</t>
+  </si>
+  <si>
+    <t>The system should clearly indicate that no matching products were found; unrelated products must not be presented as matches.</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-13.jpg</t>
   </si>
 </sst>
 </file>
@@ -2371,7 +2401,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -2400,7 +2430,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -2408,7 +2438,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -2416,10 +2446,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -2495,25 +2525,25 @@
         <v>96</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>98</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2542,25 +2572,25 @@
         <v>101</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>98</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2589,10 +2619,10 @@
         <v>105</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>106</v>
@@ -2601,13 +2631,13 @@
         <v>98</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2636,25 +2666,25 @@
         <v>110</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
@@ -2683,25 +2713,25 @@
         <v>114</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2730,10 +2760,10 @@
         <v>117</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>118</v>
@@ -2742,13 +2772,13 @@
         <v>120</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2777,25 +2807,25 @@
         <v>124</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
@@ -2827,22 +2857,22 @@
         <v>129</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2874,7 +2904,7 @@
         <v>133</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>134</v>
@@ -2883,16 +2913,16 @@
         <v>98</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>81</v>
       </c>
@@ -2921,22 +2951,30 @@
         <v>142</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="K23" s="3"/>
+        <v>547</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>548</v>
+      </c>
       <c r="L23" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-    </row>
-    <row r="24" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="M23" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="O23" s="6" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>136</v>
@@ -2948,136 +2986,160 @@
         <v>139</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G24" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="I24" s="3" t="s">
+      <c r="J24" s="3" t="s">
+        <v>550</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="J24" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="K24" s="3"/>
       <c r="L24" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
+      <c r="M24" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="O24" s="6" t="s">
+        <v>551</v>
+      </c>
     </row>
     <row r="25" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>79</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G25" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>156</v>
-      </c>
       <c r="J25" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="K25" s="3"/>
+        <v>552</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>554</v>
+      </c>
       <c r="L25" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
+      <c r="M25" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="O25" s="6" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="26" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="E26" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>102</v>
       </c>
       <c r="G26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="I26" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="H26" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>161</v>
-      </c>
       <c r="J26" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="K26" s="3"/>
+        <v>557</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>554</v>
+      </c>
       <c r="L26" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="M26" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="O26" s="6" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="27" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>77</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>166</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G27" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="J27" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="K27" s="3"/>
       <c r="L27" s="2" t="s">
@@ -3092,31 +3154,31 @@
         <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="I28" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G28" s="3" t="s">
+      <c r="J28" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>175</v>
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="2" t="s">
@@ -3131,31 +3193,31 @@
         <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="I29" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G29" s="3" t="s">
+      <c r="J29" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="2" t="s">
@@ -3170,31 +3232,31 @@
         <v>74</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>102</v>
       </c>
       <c r="G30" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="J30" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="2" t="s">
@@ -3209,31 +3271,31 @@
         <v>73</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G31" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="J31" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>195</v>
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="2" t="s">
@@ -3248,31 +3310,31 @@
         <v>72</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G32" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="J32" s="3" t="s">
         <v>198</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>201</v>
       </c>
       <c r="K32" s="3"/>
       <c r="L32" s="2" t="s">
@@ -3287,31 +3349,31 @@
         <v>71</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="I33" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G33" s="3" t="s">
+      <c r="J33" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>207</v>
       </c>
       <c r="K33" s="3"/>
       <c r="L33" s="2" t="s">
@@ -3326,31 +3388,31 @@
         <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="I34" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G34" s="3" t="s">
+      <c r="J34" s="3" t="s">
         <v>210</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>213</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="2" t="s">
@@ -3365,31 +3427,31 @@
         <v>69</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="I35" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G35" s="3" t="s">
+      <c r="J35" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>219</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="2" t="s">
@@ -3404,31 +3466,31 @@
         <v>68</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>223</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="2" t="s">
@@ -3443,31 +3505,31 @@
         <v>67</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G37" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>227</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>230</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="2" t="s">
@@ -3482,31 +3544,31 @@
         <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="I38" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G38" s="3" t="s">
+      <c r="J38" s="3" t="s">
         <v>232</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>235</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
@@ -3521,31 +3583,31 @@
         <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G39" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J39" s="3" t="s">
         <v>238</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="2" t="s">
@@ -3560,31 +3622,31 @@
         <v>64</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E40" s="2" t="s">
+      <c r="I40" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="F40" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="G40" s="3" t="s">
+      <c r="J40" s="3" t="s">
         <v>246</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
@@ -3599,31 +3661,31 @@
         <v>63</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="I41" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="G41" s="3" t="s">
+      <c r="J41" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="2" t="s">
@@ -3638,31 +3700,31 @@
         <v>62</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="I42" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="G42" s="3" t="s">
+      <c r="J42" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>261</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="2" t="s">
@@ -3677,31 +3739,31 @@
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="I43" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="G43" s="3" t="s">
+      <c r="J43" s="3" t="s">
         <v>264</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="J43" s="3" t="s">
-        <v>267</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="2" t="s">
@@ -3716,31 +3778,31 @@
         <v>60</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="I44" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="G44" s="3" t="s">
+      <c r="J44" s="3" t="s">
         <v>270</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="J44" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="K44" s="3"/>
       <c r="L44" s="2" t="s">
@@ -3755,31 +3817,31 @@
         <v>59</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="H45" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E45" s="2" t="s">
+      <c r="I45" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="F45" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="G45" s="3" t="s">
+      <c r="J45" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="J45" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="2" t="s">
@@ -3794,31 +3856,31 @@
         <v>58</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J46" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>283</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="J46" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="K46" s="3"/>
       <c r="L46" s="2" t="s">
@@ -3833,31 +3895,31 @@
         <v>57</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="I47" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G47" s="3" t="s">
+      <c r="J47" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="H47" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="I47" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="J47" s="3" t="s">
-        <v>294</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="2" t="s">
@@ -3872,31 +3934,31 @@
         <v>56</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="2" t="s">
@@ -3911,31 +3973,31 @@
         <v>55</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="J49" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="G49" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="H49" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="I49" s="3" t="s">
-        <v>302</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>303</v>
       </c>
       <c r="K49" s="3"/>
       <c r="L49" s="2" t="s">
@@ -3950,31 +4012,31 @@
         <v>54</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="H50" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="C50" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E50" s="2" t="s">
+      <c r="I50" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="F50" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="G50" s="3" t="s">
+      <c r="J50" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="J50" s="3" t="s">
-        <v>311</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="2" t="s">
@@ -3989,31 +4051,31 @@
         <v>53</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>102</v>
       </c>
       <c r="G51" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="J51" s="3" t="s">
         <v>315</v>
-      </c>
-      <c r="H51" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="I51" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="J51" s="3" t="s">
-        <v>318</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="2" t="s">
@@ -4028,31 +4090,31 @@
         <v>52</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="I52" s="3" t="s">
         <v>319</v>
       </c>
-      <c r="C52" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G52" s="3" t="s">
+      <c r="J52" s="3" t="s">
         <v>320</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="J52" s="3" t="s">
-        <v>323</v>
       </c>
       <c r="K52" s="3"/>
       <c r="L52" s="2" t="s">
@@ -4067,31 +4129,31 @@
         <v>51</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>325</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>328</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G53" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="J53" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>330</v>
-      </c>
-      <c r="I53" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="J53" s="3" t="s">
-        <v>332</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="2" t="s">
@@ -4106,31 +4168,31 @@
         <v>50</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="I54" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>326</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G54" s="3" t="s">
+      <c r="J54" s="3" t="s">
         <v>335</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="J54" s="3" t="s">
-        <v>338</v>
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="2" t="s">
@@ -4145,31 +4207,31 @@
         <v>49</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E55" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>342</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G55" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="J55" s="3" t="s">
         <v>343</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="I55" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="J55" s="3" t="s">
-        <v>346</v>
       </c>
       <c r="K55" s="3"/>
       <c r="L55" s="2" t="s">
@@ -4184,31 +4246,31 @@
         <v>48</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="I56" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="C56" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G56" s="3" t="s">
+      <c r="J56" s="3" t="s">
         <v>348</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>350</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>351</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="2" t="s">
@@ -4223,31 +4285,31 @@
         <v>47</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="I57" s="3" t="s">
         <v>353</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G57" s="3" t="s">
+      <c r="J57" s="3" t="s">
         <v>354</v>
-      </c>
-      <c r="H57" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="J57" s="3" t="s">
-        <v>357</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="2" t="s">
@@ -4262,31 +4324,31 @@
         <v>46</v>
       </c>
       <c r="B58" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="I58" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="G58" s="3" t="s">
+      <c r="J58" s="3" t="s">
         <v>359</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="J58" s="3" t="s">
-        <v>362</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="2" t="s">
@@ -4301,31 +4363,31 @@
         <v>45</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="I59" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G59" s="3" t="s">
+      <c r="J59" s="3" t="s">
         <v>365</v>
-      </c>
-      <c r="H59" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>367</v>
-      </c>
-      <c r="J59" s="3" t="s">
-        <v>368</v>
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="2" t="s">
@@ -4340,31 +4402,31 @@
         <v>44</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="I60" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G60" s="3" t="s">
+      <c r="J60" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>371</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>372</v>
-      </c>
-      <c r="J60" s="3" t="s">
-        <v>373</v>
       </c>
       <c r="K60" s="3"/>
       <c r="L60" s="2" t="s">
@@ -4379,31 +4441,31 @@
         <v>43</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="I61" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="D61" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="G61" s="3" t="s">
+      <c r="J61" s="3" t="s">
         <v>376</v>
-      </c>
-      <c r="H61" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="I61" s="3" t="s">
-        <v>378</v>
-      </c>
-      <c r="J61" s="3" t="s">
-        <v>379</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="2" t="s">
@@ -4418,31 +4480,31 @@
         <v>42</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="J62" s="3" t="s">
         <v>381</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>382</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="J62" s="3" t="s">
-        <v>384</v>
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="2" t="s">
@@ -4457,31 +4519,31 @@
         <v>41</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>384</v>
+      </c>
+      <c r="I63" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="C63" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G63" s="3" t="s">
+      <c r="J63" s="3" t="s">
         <v>386</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="I63" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="J63" s="3" t="s">
-        <v>389</v>
       </c>
       <c r="K63" s="3"/>
       <c r="L63" s="2" t="s">
@@ -4496,31 +4558,31 @@
         <v>40</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>391</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>394</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G64" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="J64" s="3" t="s">
         <v>395</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="I64" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="J64" s="3" t="s">
-        <v>398</v>
       </c>
       <c r="K64" s="3"/>
       <c r="L64" s="2" t="s">
@@ -4535,31 +4597,31 @@
         <v>39</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>392</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="J65" s="3" t="s">
         <v>399</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>392</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>400</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="J65" s="3" t="s">
-        <v>402</v>
       </c>
       <c r="K65" s="3"/>
       <c r="L65" s="2" t="s">
@@ -4574,31 +4636,31 @@
         <v>38</v>
       </c>
       <c r="B66" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="H66" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>404</v>
-      </c>
-      <c r="E66" s="2" t="s">
+      <c r="I66" s="3" t="s">
         <v>406</v>
       </c>
-      <c r="F66" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="G66" s="3" t="s">
+      <c r="J66" s="3" t="s">
         <v>407</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>410</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="2" t="s">
@@ -4613,31 +4675,31 @@
         <v>37</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H67" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="C67" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="E67" s="2" t="s">
+      <c r="I67" s="3" t="s">
         <v>415</v>
       </c>
-      <c r="F67" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="G67" s="3" t="s">
+      <c r="J67" s="3" t="s">
         <v>416</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>417</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>419</v>
       </c>
       <c r="K67" s="3"/>
       <c r="L67" s="2" t="s">
@@ -4646,7 +4708,7 @@
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="68" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4654,13 +4716,13 @@
         <v>36</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>119</v>
@@ -4669,16 +4731,16 @@
         <v>135</v>
       </c>
       <c r="G68" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="J68" s="3" t="s">
         <v>424</v>
-      </c>
-      <c r="H68" s="3" t="s">
-        <v>425</v>
-      </c>
-      <c r="I68" s="3" t="s">
-        <v>426</v>
-      </c>
-      <c r="J68" s="3" t="s">
-        <v>427</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="2" t="s">
@@ -4693,13 +4755,13 @@
         <v>35</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>119</v>
@@ -4708,16 +4770,16 @@
         <v>135</v>
       </c>
       <c r="G69" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="J69" s="3" t="s">
         <v>429</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>430</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>431</v>
-      </c>
-      <c r="J69" s="3" t="s">
-        <v>432</v>
       </c>
       <c r="K69" s="3"/>
       <c r="L69" s="2" t="s">
@@ -4732,31 +4794,31 @@
         <v>34</v>
       </c>
       <c r="B70" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="H70" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="C70" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="E70" s="2" t="s">
+      <c r="I70" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="F70" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="G70" s="3" t="s">
+      <c r="J70" s="3" t="s">
         <v>437</v>
-      </c>
-      <c r="H70" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="J70" s="3" t="s">
-        <v>440</v>
       </c>
       <c r="K70" s="3"/>
       <c r="L70" s="2" t="s">
@@ -4771,31 +4833,31 @@
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="H71" s="3" t="s">
         <v>444</v>
       </c>
-      <c r="C71" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="E71" s="2" t="s">
+      <c r="I71" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="F71" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="G71" s="3" t="s">
+      <c r="J71" s="3" t="s">
         <v>446</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>447</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>448</v>
-      </c>
-      <c r="J71" s="3" t="s">
-        <v>449</v>
       </c>
       <c r="K71" s="3"/>
       <c r="L71" s="2" t="s">
@@ -4810,31 +4872,31 @@
         <v>32</v>
       </c>
       <c r="B72" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="I72" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="C72" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>443</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="G72" s="3" t="s">
+      <c r="J72" s="3" t="s">
         <v>453</v>
-      </c>
-      <c r="H72" s="3" t="s">
-        <v>454</v>
-      </c>
-      <c r="I72" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="J72" s="3" t="s">
-        <v>456</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="2" t="s">
@@ -4849,31 +4911,31 @@
         <v>31</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="H73" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="E73" s="2" t="s">
+      <c r="I73" s="3" t="s">
         <v>461</v>
       </c>
-      <c r="F73" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="G73" s="3" t="s">
+      <c r="J73" s="3" t="s">
         <v>462</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>463</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="J73" s="3" t="s">
-        <v>465</v>
       </c>
       <c r="K73" s="3"/>
       <c r="L73" s="2" t="s">
@@ -4888,31 +4950,31 @@
         <v>30</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="H74" s="3" t="s">
         <v>467</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E74" s="2" t="s">
+      <c r="I74" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="F74" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="G74" s="3" t="s">
+      <c r="J74" s="3" t="s">
         <v>469</v>
-      </c>
-      <c r="H74" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="I74" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="J74" s="3" t="s">
-        <v>472</v>
       </c>
       <c r="K74" s="3"/>
       <c r="L74" s="2" t="s">
@@ -4921,7 +4983,7 @@
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="75" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
@@ -4929,31 +4991,31 @@
         <v>29</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="I75" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="G75" s="3" t="s">
+      <c r="J75" s="3" t="s">
         <v>477</v>
-      </c>
-      <c r="H75" s="3" t="s">
-        <v>478</v>
-      </c>
-      <c r="I75" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="J75" s="3" t="s">
-        <v>480</v>
       </c>
       <c r="K75" s="3"/>
       <c r="L75" s="2" t="s">
@@ -4962,7 +5024,7 @@
       <c r="M75" s="2"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -4970,31 +5032,31 @@
         <v>28</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="H76" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E76" s="2" t="s">
+      <c r="I76" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="F76" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="G76" s="3" t="s">
+      <c r="J76" s="3" t="s">
         <v>486</v>
-      </c>
-      <c r="H76" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="I76" s="3" t="s">
-        <v>488</v>
-      </c>
-      <c r="J76" s="3" t="s">
-        <v>489</v>
       </c>
       <c r="K76" s="3"/>
       <c r="L76" s="2" t="s">
@@ -5003,7 +5065,7 @@
       <c r="M76" s="2"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -5011,31 +5073,31 @@
         <v>27</v>
       </c>
       <c r="B77" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="I77" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>523</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="F77" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="G77" s="3" t="s">
+      <c r="J77" s="3" t="s">
         <v>494</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>495</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="J77" s="3" t="s">
-        <v>497</v>
       </c>
       <c r="K77" s="3"/>
       <c r="L77" s="2" t="s">
@@ -5050,31 +5112,31 @@
         <v>26</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="H78" s="3" t="s">
         <v>500</v>
       </c>
-      <c r="C78" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="E78" s="2" t="s">
+      <c r="I78" s="3" t="s">
         <v>501</v>
       </c>
-      <c r="F78" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="G78" s="3" t="s">
+      <c r="J78" s="3" t="s">
         <v>502</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="I78" s="3" t="s">
-        <v>504</v>
-      </c>
-      <c r="J78" s="3" t="s">
-        <v>505</v>
       </c>
       <c r="K78" s="3"/>
       <c r="L78" s="2" t="s">
@@ -5089,31 +5151,31 @@
         <v>25</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="H79" s="3" t="s">
         <v>507</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="D79" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="E79" s="2" t="s">
+      <c r="I79" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="F79" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="G79" s="3" t="s">
+      <c r="J79" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>510</v>
-      </c>
-      <c r="I79" s="3" t="s">
-        <v>511</v>
-      </c>
-      <c r="J79" s="3" t="s">
-        <v>512</v>
       </c>
       <c r="K79" s="3"/>
       <c r="L79" s="2" t="s">
@@ -5136,11 +5198,15 @@
     <hyperlink ref="O20" r:id="rId8" xr:uid="{F5787B2D-5828-4623-8A64-5D9CFF9E641B}"/>
     <hyperlink ref="O21" r:id="rId9" xr:uid="{D4758FBB-2393-4158-82C5-88B1B57F3D54}"/>
     <hyperlink ref="O22" r:id="rId10" xr:uid="{046CBEDE-BA76-4650-974F-62FAF5F2D2F7}"/>
+    <hyperlink ref="O23" r:id="rId11" xr:uid="{616974E5-44EC-448E-875A-A3503AB3FF1C}"/>
+    <hyperlink ref="O24" r:id="rId12" xr:uid="{2B998C3F-3E9D-4783-BF1E-B571D6980D52}"/>
+    <hyperlink ref="O25" r:id="rId13" xr:uid="{A9F91156-7544-416B-BABA-57F820D7A096}"/>
+    <hyperlink ref="O26" r:id="rId14" xr:uid="{3F9B958A-D6BB-42DD-A59A-8097230A06A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId11"/>
-    <tablePart r:id="rId12"/>
+    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updating Document and Execute test cases 14-20
</commit_message>
<xml_diff>
--- a/04-Test_Cases/01-Test_Cases.xlsx
+++ b/04-Test_Cases/01-Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\QADemo E-Commerce Application Manual Testing\QADemoE-CommerceApplicationManualTesting\04-Test_Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71B03D3-63A4-45DC-A51D-7BADAD0CC11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D32DD462-46C2-4C36-98A4-1E2462C1449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="574">
   <si>
     <t>Key</t>
   </si>
@@ -549,11 +549,6 @@
     <t>At least one available product is listed.</t>
   </si>
   <si>
-    <t>1. Select a product from the listing.
-2. Open its details page or panel.
-3. Review the displayed information.</t>
-  </si>
-  <si>
     <t>An available product.</t>
   </si>
   <si>
@@ -566,12 +561,6 @@
     <t>At least two products with distinguishable descriptions are available.</t>
   </si>
   <si>
-    <t>1. Open Product A details and record its description.
-2. Return to the listing.
-3. Open Product B details.
-4. Compare the displayed description with each selected product.</t>
-  </si>
-  <si>
     <t>Two products with different descriptions.</t>
   </si>
   <si>
@@ -588,10 +577,6 @@
   </si>
   <si>
     <t>An available product exists.</t>
-  </si>
-  <si>
-    <t>1. Open the product details.
-2. Inspect price and availability/status information.</t>
   </si>
   <si>
     <t>Available product.</t>
@@ -632,11 +617,6 @@
     <t>A customer is on the product listing/details page and an eligible product is available.</t>
   </si>
   <si>
-    <t>1. Select an eligible product.
-2. Click Add to Cart.
-3. Open the cart or inspect the cart indicator.</t>
-  </si>
-  <si>
     <t>One eligible product, quantity 1.</t>
   </si>
   <si>
@@ -652,15 +632,6 @@
     <t>At least two eligible products are available.</t>
   </si>
   <si>
-    <t>1. Add Product A to the cart.
-2. Return to the listing.
-3. Add Product B.
-4. Open the cart.</t>
-  </si>
-  <si>
-    <t>Product A and Product B.</t>
-  </si>
-  <si>
     <t>Both selected products appear in the cart with the correct identities and quantities.</t>
   </si>
   <si>
@@ -671,11 +642,6 @@
   </si>
   <si>
     <t>An eligible product is available and the cart is initially empty.</t>
-  </si>
-  <si>
-    <t>1. Add the same product to the cart.
-2. Return to the product and add it again.
-3. Open the cart and inspect item rows and quantities.</t>
   </si>
   <si>
     <t>Same product added twice.</t>
@@ -1856,6 +1822,81 @@
   </si>
   <si>
     <t>..\Evidence\TC-13.jpg</t>
+  </si>
+  <si>
+    <t>1. Select a product from the listing.
+2. Open its details page.
+3. Review the displayed information.</t>
+  </si>
+  <si>
+    <t>The product details should be easily accessible and the information displayed must correspond to the selected product.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-14.jpg</t>
+  </si>
+  <si>
+    <t>1. Open Product-1 details and record its description.
+2. Return to the listing.
+3. Open Product-2 details.
+4. Compare the displayed description with each selected product.</t>
+  </si>
+  <si>
+    <t>The detailed information view for each product should display only the details related to that specific product; it should not include information about any other product.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-15.jpg</t>
+  </si>
+  <si>
+    <t>1. Open the product details.
+2. Inspect price and availability information.</t>
+  </si>
+  <si>
+    <t>The current product price and applicable availability information should be displayed clearly.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-16.jpg</t>
+  </si>
+  <si>
+    <t>The product should be clearly marked unavailable and an ineligible purchase action should be prevented.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-17.jpg</t>
+  </si>
+  <si>
+    <t>1. Select an eligible product.
+2. Click Add to Cart.
+3. Inspect the cart indicator.</t>
+  </si>
+  <si>
+    <t>The selected product should be added to the cart and the cart should reflect the addition.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-18.jpg</t>
+  </si>
+  <si>
+    <t>1. Add Product-1 to the cart.
+2. Return to the listing.
+3. Add Product-2.
+4. Open the cart.</t>
+  </si>
+  <si>
+    <t>Product-1 and Product-2.</t>
+  </si>
+  <si>
+    <t>Both selected should product appear in the cart with the correct identities and quantities.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-19.jpg</t>
+  </si>
+  <si>
+    <t>1. Add the same product to the cart two times.
+2. Open the cart and inspect item rows and quantities.</t>
+  </si>
+  <si>
+    <t>The cart should handle repeated additions consistently with the application’s defined behavior; product count/quantity and totals must be accurate without unintended duplicate or lost items.</t>
+  </si>
+  <si>
+    <t>..\Evidence\TC-20.jpg</t>
   </si>
 </sst>
 </file>
@@ -1939,7 +1980,21 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2057,6 +2112,12 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF9999"/>
+      <color rgb="FFFFCCCC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2069,35 +2130,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC0972E8-E27C-45A1-BD68-74AC7D938AB0}" name="Table13" displayName="Table13" ref="A2:B9" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AC0972E8-E27C-45A1-BD68-74AC7D938AB0}" name="Table13" displayName="Table13" ref="A2:B9" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A2:B9" xr:uid="{AC0972E8-E27C-45A1-BD68-74AC7D938AB0}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{05A7F6E6-1E8F-4B9C-810B-C9396C6B5456}" name="Key" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{FFC49D79-8BCB-4241-9F71-306E1E028408}" name="Value" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{05A7F6E6-1E8F-4B9C-810B-C9396C6B5456}" name="Key" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{FFC49D79-8BCB-4241-9F71-306E1E028408}" name="Value" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}" name="Table2" displayName="Table2" ref="A13:O79" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}" name="Table2" displayName="Table2" ref="A13:O79" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A13:O79" xr:uid="{0069FDD6-BA15-40E1-A10B-744F07A0EA08}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D243436B-E280-47D1-9048-A55E41BCCDA7}" name="Test Case ID" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{04E3F4CC-C517-4D34-AF59-7D35761EA7A2}" name="Test Case Title" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{B5CDD440-C8DB-4010-81FA-5ED0AE5FAC24}" name="Test Scenario ID" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{A2E98623-58F2-4087-AA4D-768C17D712B4}" name="Requirements ID" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{0948D040-2ED0-49D3-A3F7-D2DE67922DAC}" name="Module" dataDxfId="10"/>
-    <tableColumn id="20" xr3:uid="{4C1A7320-75FB-4DC9-B451-C7A962DC6823}" name="Test Type" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{7DAE9DF7-AED9-4464-B6F3-1D0B5E71B685}" name="Preconditions" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{6563B834-3510-45D1-A3BB-261DAA503DC2}" name="Test Steps" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{8A9D41F2-3075-43D5-9FCE-201D9AE235D8}" name="Test Data" dataDxfId="6"/>
-    <tableColumn id="19" xr3:uid="{C0B5DD96-4C37-470C-A90B-C0F6BAEE4561}" name="Expected Result" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{EBECA87A-F936-442B-813B-CB8A8FF2959A}" name="Actual Result" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{CE5B88B8-BB15-458C-8434-70F85E2E87E6}" name="Priority" dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{C38F7409-03E4-49EE-B8AB-36C447EA718E}" name="Execution Status" dataDxfId="2"/>
-    <tableColumn id="15" xr3:uid="{3F9ED411-BFCC-43BC-9869-C0177649C0FB}" name="Defect ID" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{94FF1D6A-77E0-4094-9426-C2A41DEB43DF}" name="Remarks / Evidence" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D243436B-E280-47D1-9048-A55E41BCCDA7}" name="Test Case ID" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{04E3F4CC-C517-4D34-AF59-7D35761EA7A2}" name="Test Case Title" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{B5CDD440-C8DB-4010-81FA-5ED0AE5FAC24}" name="Test Scenario ID" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{A2E98623-58F2-4087-AA4D-768C17D712B4}" name="Requirements ID" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{0948D040-2ED0-49D3-A3F7-D2DE67922DAC}" name="Module" dataDxfId="12"/>
+    <tableColumn id="20" xr3:uid="{4C1A7320-75FB-4DC9-B451-C7A962DC6823}" name="Test Type" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{7DAE9DF7-AED9-4464-B6F3-1D0B5E71B685}" name="Preconditions" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{6563B834-3510-45D1-A3BB-261DAA503DC2}" name="Test Steps" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{8A9D41F2-3075-43D5-9FCE-201D9AE235D8}" name="Test Data" dataDxfId="8"/>
+    <tableColumn id="19" xr3:uid="{C0B5DD96-4C37-470C-A90B-C0F6BAEE4561}" name="Expected Result" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{EBECA87A-F936-442B-813B-CB8A8FF2959A}" name="Actual Result" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{CE5B88B8-BB15-458C-8434-70F85E2E87E6}" name="Priority" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{C38F7409-03E4-49EE-B8AB-36C447EA718E}" name="Execution Status" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{3F9ED411-BFCC-43BC-9869-C0177649C0FB}" name="Defect ID" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{94FF1D6A-77E0-4094-9426-C2A41DEB43DF}" name="Remarks / Evidence" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium25" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2375,11 +2436,11 @@
     <col min="4" max="4" width="19.88671875" customWidth="1"/>
     <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="34.77734375" customWidth="1"/>
+    <col min="7" max="7" width="36.44140625" customWidth="1"/>
+    <col min="8" max="8" width="37.88671875" customWidth="1"/>
     <col min="9" max="9" width="30.6640625" customWidth="1"/>
-    <col min="10" max="10" width="34.44140625" customWidth="1"/>
-    <col min="11" max="11" width="34.5546875" customWidth="1"/>
+    <col min="10" max="10" width="35.109375" customWidth="1"/>
+    <col min="11" max="11" width="36.21875" customWidth="1"/>
     <col min="12" max="12" width="20.109375" customWidth="1"/>
     <col min="13" max="13" width="20.33203125" customWidth="1"/>
     <col min="14" max="14" width="21.77734375" customWidth="1"/>
@@ -2401,7 +2462,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
@@ -2430,7 +2491,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>9</v>
@@ -2438,7 +2499,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>9</v>
@@ -2446,10 +2507,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -2525,25 +2586,25 @@
         <v>96</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>98</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2572,25 +2633,25 @@
         <v>101</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>98</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2619,10 +2680,10 @@
         <v>105</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>106</v>
@@ -2631,13 +2692,13 @@
         <v>98</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N16" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O16" s="6" t="s">
         <v>520</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2666,25 +2727,25 @@
         <v>110</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
@@ -2713,25 +2774,25 @@
         <v>114</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -2760,10 +2821,10 @@
         <v>117</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>536</v>
+        <v>529</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>118</v>
@@ -2772,13 +2833,13 @@
         <v>120</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2807,25 +2868,25 @@
         <v>124</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>538</v>
+        <v>531</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>539</v>
+        <v>532</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>540</v>
+        <v>533</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>541</v>
+        <v>534</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
@@ -2857,22 +2918,22 @@
         <v>129</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>542</v>
+        <v>535</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>543</v>
+        <v>536</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>112</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O21" s="6" t="s">
-        <v>544</v>
+        <v>537</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2904,7 +2965,7 @@
         <v>133</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>545</v>
+        <v>538</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>134</v>
@@ -2913,13 +2974,13 @@
         <v>98</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
@@ -2951,22 +3012,22 @@
         <v>142</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>547</v>
+        <v>540</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>548</v>
+        <v>541</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>98</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O23" s="6" t="s">
-        <v>549</v>
+        <v>542</v>
       </c>
     </row>
     <row r="24" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -2998,7 +3059,7 @@
         <v>146</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>550</v>
+        <v>543</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>147</v>
@@ -3007,13 +3068,13 @@
         <v>112</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="72" x14ac:dyDescent="0.3">
@@ -3045,22 +3106,22 @@
         <v>155</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>120</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="O25" s="6" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
     </row>
     <row r="26" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
@@ -3092,25 +3153,25 @@
         <v>159</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>120</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>77</v>
       </c>
@@ -3133,28 +3194,36 @@
         <v>164</v>
       </c>
       <c r="H27" s="3" t="s">
+        <v>553</v>
+      </c>
+      <c r="I27" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="I27" s="3" t="s">
+      <c r="J27" s="3" t="s">
+        <v>554</v>
+      </c>
+      <c r="K27" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="J27" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="K27" s="3"/>
       <c r="L27" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
+      <c r="M27" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O27" s="6" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="28" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>160</v>
@@ -3166,37 +3235,45 @@
         <v>163</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G28" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="I28" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="J28" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="K28" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="I28" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="J28" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="K28" s="3"/>
       <c r="L28" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
+      <c r="M28" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="29" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>161</v>
@@ -3208,34 +3285,42 @@
         <v>148</v>
       </c>
       <c r="G29" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>559</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>560</v>
+      </c>
+      <c r="K29" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H29" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="K29" s="3"/>
       <c r="L29" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
+      <c r="M29" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O29" s="6" t="s">
+        <v>561</v>
+      </c>
     </row>
     <row r="30" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>161</v>
@@ -3247,172 +3332,204 @@
         <v>102</v>
       </c>
       <c r="G30" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>562</v>
+      </c>
+      <c r="K30" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="H30" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="K30" s="3"/>
       <c r="L30" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-    </row>
-    <row r="31" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="M30" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O30" s="6" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>185</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>190</v>
+        <v>564</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="K31" s="3"/>
+        <v>565</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>188</v>
+      </c>
       <c r="L31" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+      <c r="M31" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O31" s="6" t="s">
+        <v>566</v>
+      </c>
     </row>
     <row r="32" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>196</v>
+        <v>567</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>197</v>
+        <v>568</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="K32" s="3"/>
+        <v>569</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>192</v>
+      </c>
       <c r="L32" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
+      <c r="M32" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O32" s="6" t="s">
+        <v>570</v>
+      </c>
     </row>
     <row r="33" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>148</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>202</v>
+        <v>571</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="K33" s="3"/>
+        <v>572</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>197</v>
+      </c>
       <c r="L33" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
+      <c r="M33" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O33" s="6" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="34" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="K34" s="3"/>
       <c r="L34" s="2" t="s">
@@ -3427,31 +3544,31 @@
         <v>69</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>148</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="2" t="s">
@@ -3466,31 +3583,31 @@
         <v>68</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="H36" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="G36" s="3" t="s">
+      <c r="I36" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>213</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>220</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="2" t="s">
@@ -3505,31 +3622,31 @@
         <v>67</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="2" t="s">
@@ -3544,31 +3661,31 @@
         <v>66</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G38" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>229</v>
-      </c>
       <c r="H38" s="3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="2" t="s">
@@ -3583,31 +3700,31 @@
         <v>65</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="2" t="s">
@@ -3622,31 +3739,31 @@
         <v>64</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="J40" s="3" t="s">
         <v>239</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>246</v>
       </c>
       <c r="K40" s="3"/>
       <c r="L40" s="2" t="s">
@@ -3661,31 +3778,31 @@
         <v>63</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="G41" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>249</v>
-      </c>
       <c r="H41" s="3" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="K41" s="3"/>
       <c r="L41" s="2" t="s">
@@ -3700,31 +3817,31 @@
         <v>62</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D42" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="E42" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>247</v>
-      </c>
       <c r="G42" s="3" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="K42" s="3"/>
       <c r="L42" s="2" t="s">
@@ -3739,31 +3856,31 @@
         <v>61</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="K43" s="3"/>
       <c r="L43" s="2" t="s">
@@ -3773,36 +3890,36 @@
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
     </row>
-    <row r="44" spans="1:15" ht="72" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="K44" s="3"/>
       <c r="L44" s="2" t="s">
@@ -3812,36 +3929,36 @@
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
-    <row r="45" spans="1:15" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="J45" s="3" t="s">
         <v>271</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>272</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="H45" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="J45" s="3" t="s">
-        <v>278</v>
       </c>
       <c r="K45" s="3"/>
       <c r="L45" s="2" t="s">
@@ -3856,31 +3973,31 @@
         <v>58</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="K46" s="3"/>
       <c r="L46" s="2" t="s">
@@ -3895,31 +4012,31 @@
         <v>57</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="K47" s="3"/>
       <c r="L47" s="2" t="s">
@@ -3934,31 +4051,31 @@
         <v>56</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G48" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="I48" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="H48" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>295</v>
-      </c>
       <c r="J48" s="3" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="K48" s="3"/>
       <c r="L48" s="2" t="s">
@@ -3973,31 +4090,31 @@
         <v>55</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="K49" s="3"/>
       <c r="L49" s="2" t="s">
@@ -4007,36 +4124,36 @@
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
     </row>
-    <row r="50" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="J50" s="3" t="s">
         <v>301</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="J50" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="K50" s="3"/>
       <c r="L50" s="2" t="s">
@@ -4051,31 +4168,31 @@
         <v>53</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>102</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="I51" s="3" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="K51" s="3"/>
       <c r="L51" s="2" t="s">
@@ -4090,31 +4207,31 @@
         <v>52</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="K52" s="3"/>
       <c r="L52" s="2" t="s">
@@ -4129,31 +4246,31 @@
         <v>51</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="K53" s="3"/>
       <c r="L53" s="2" t="s">
@@ -4168,31 +4285,31 @@
         <v>50</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="E54" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G54" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="F54" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>332</v>
-      </c>
       <c r="H54" s="3" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="2" t="s">
@@ -4207,31 +4324,31 @@
         <v>49</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>97</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="I55" s="3" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="K55" s="3"/>
       <c r="L55" s="2" t="s">
@@ -4246,31 +4363,31 @@
         <v>48</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E56" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="H56" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="F56" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>346</v>
-      </c>
       <c r="I56" s="3" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="J56" s="3" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="2" t="s">
@@ -4280,36 +4397,36 @@
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
     </row>
-    <row r="57" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="I57" s="3" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="J57" s="3" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="2" t="s">
@@ -4324,31 +4441,31 @@
         <v>46</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="G58" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>356</v>
-      </c>
       <c r="H58" s="3" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="I58" s="3" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="2" t="s">
@@ -4363,31 +4480,31 @@
         <v>45</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>362</v>
+        <v>355</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>363</v>
+        <v>356</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="J59" s="3" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="2" t="s">
@@ -4402,31 +4519,31 @@
         <v>44</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="G60" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>367</v>
-      </c>
       <c r="H60" s="3" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="I60" s="3" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="J60" s="3" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="K60" s="3"/>
       <c r="L60" s="2" t="s">
@@ -4436,36 +4553,36 @@
       <c r="N60" s="2"/>
       <c r="O60" s="2"/>
     </row>
-    <row r="61" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="I61" s="3" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="J61" s="3" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
       <c r="K61" s="3"/>
       <c r="L61" s="2" t="s">
@@ -4480,31 +4597,31 @@
         <v>42</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>148</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="I62" s="3" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="2" t="s">
@@ -4514,36 +4631,36 @@
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
     </row>
-    <row r="63" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="H63" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="D63" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>383</v>
-      </c>
-      <c r="H63" s="3" t="s">
-        <v>384</v>
-      </c>
       <c r="I63" s="3" t="s">
-        <v>385</v>
+        <v>378</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>386</v>
+        <v>379</v>
       </c>
       <c r="K63" s="3"/>
       <c r="L63" s="2" t="s">
@@ -4558,31 +4675,31 @@
         <v>40</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>391</v>
+        <v>384</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>392</v>
+        <v>385</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="I64" s="3" t="s">
-        <v>394</v>
+        <v>387</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>395</v>
+        <v>388</v>
       </c>
       <c r="K64" s="3"/>
       <c r="L64" s="2" t="s">
@@ -4597,31 +4714,31 @@
         <v>39</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>396</v>
+        <v>389</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>388</v>
+        <v>381</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>389</v>
+        <v>382</v>
       </c>
       <c r="E65" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="I65" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="F65" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="G65" s="3" t="s">
+      <c r="J65" s="3" t="s">
         <v>392</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="I65" s="3" t="s">
-        <v>398</v>
-      </c>
-      <c r="J65" s="3" t="s">
-        <v>399</v>
       </c>
       <c r="K65" s="3"/>
       <c r="L65" s="2" t="s">
@@ -4631,36 +4748,36 @@
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
     </row>
-    <row r="66" spans="1:15" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>398</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="J66" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>401</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>407</v>
       </c>
       <c r="K66" s="3"/>
       <c r="L66" s="2" t="s">
@@ -4670,36 +4787,36 @@
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
     </row>
-    <row r="67" spans="1:15" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>411</v>
+        <v>404</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="J67" s="3" t="s">
         <v>409</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="I67" s="3" t="s">
-        <v>415</v>
-      </c>
-      <c r="J67" s="3" t="s">
-        <v>416</v>
       </c>
       <c r="K67" s="3"/>
       <c r="L67" s="2" t="s">
@@ -4708,21 +4825,21 @@
       <c r="M67" s="2"/>
       <c r="N67" s="2"/>
       <c r="O67" s="2" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>119</v>
@@ -4731,16 +4848,16 @@
         <v>135</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="I68" s="3" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="K68" s="3"/>
       <c r="L68" s="2" t="s">
@@ -4750,18 +4867,18 @@
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
     </row>
-    <row r="69" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>425</v>
+        <v>418</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>418</v>
+        <v>411</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>419</v>
+        <v>412</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>119</v>
@@ -4770,16 +4887,16 @@
         <v>135</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>426</v>
+        <v>419</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="I69" s="3" t="s">
-        <v>428</v>
+        <v>421</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>429</v>
+        <v>422</v>
       </c>
       <c r="K69" s="3"/>
       <c r="L69" s="2" t="s">
@@ -4794,31 +4911,31 @@
         <v>34</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>432</v>
+        <v>425</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="J70" s="3" t="s">
         <v>430</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>434</v>
-      </c>
-      <c r="H70" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="I70" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="J70" s="3" t="s">
-        <v>437</v>
       </c>
       <c r="K70" s="3"/>
       <c r="L70" s="2" t="s">
@@ -4833,31 +4950,31 @@
         <v>33</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="C71" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>437</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="J71" s="3" t="s">
         <v>439</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>440</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>442</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>443</v>
-      </c>
-      <c r="H71" s="3" t="s">
-        <v>444</v>
-      </c>
-      <c r="I71" s="3" t="s">
-        <v>445</v>
-      </c>
-      <c r="J71" s="3" t="s">
-        <v>446</v>
       </c>
       <c r="K71" s="3"/>
       <c r="L71" s="2" t="s">
@@ -4872,31 +4989,31 @@
         <v>32</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>440</v>
+        <v>433</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>442</v>
+        <v>435</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="I72" s="3" t="s">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>453</v>
+        <v>446</v>
       </c>
       <c r="K72" s="3"/>
       <c r="L72" s="2" t="s">
@@ -4911,31 +5028,31 @@
         <v>31</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>457</v>
+        <v>450</v>
       </c>
       <c r="C73" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="J73" s="3" t="s">
         <v>455</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>460</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>461</v>
-      </c>
-      <c r="J73" s="3" t="s">
-        <v>462</v>
       </c>
       <c r="K73" s="3"/>
       <c r="L73" s="2" t="s">
@@ -4950,31 +5067,31 @@
         <v>30</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
       <c r="C74" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="F74" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="D74" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>470</v>
-      </c>
       <c r="G74" s="3" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="I74" s="3" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="K74" s="3"/>
       <c r="L74" s="2" t="s">
@@ -4983,39 +5100,39 @@
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
       <c r="O74" s="2" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="75" spans="1:15" ht="100.8" x14ac:dyDescent="0.3">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" ht="72" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="I75" s="3" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="J75" s="3" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="K75" s="3"/>
       <c r="L75" s="2" t="s">
@@ -5024,7 +5141,7 @@
       <c r="M75" s="2"/>
       <c r="N75" s="2"/>
       <c r="O75" s="2" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
     </row>
     <row r="76" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -5032,31 +5149,31 @@
         <v>28</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="C76" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="F76" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>487</v>
-      </c>
       <c r="G76" s="3" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="I76" s="3" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="J76" s="3" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
       <c r="K76" s="3"/>
       <c r="L76" s="2" t="s">
@@ -5065,7 +5182,7 @@
       <c r="M76" s="2"/>
       <c r="N76" s="2"/>
       <c r="O76" s="2" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
     </row>
     <row r="77" spans="1:15" ht="86.4" x14ac:dyDescent="0.3">
@@ -5073,31 +5190,31 @@
         <v>27</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="F77" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="J77" s="3" t="s">
         <v>487</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="H77" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>493</v>
-      </c>
-      <c r="J77" s="3" t="s">
-        <v>494</v>
       </c>
       <c r="K77" s="3"/>
       <c r="L77" s="2" t="s">
@@ -5112,31 +5229,31 @@
         <v>26</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="J78" s="3" t="s">
         <v>495</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="G78" s="3" t="s">
-        <v>499</v>
-      </c>
-      <c r="H78" s="3" t="s">
-        <v>500</v>
-      </c>
-      <c r="I78" s="3" t="s">
-        <v>501</v>
-      </c>
-      <c r="J78" s="3" t="s">
-        <v>502</v>
       </c>
       <c r="K78" s="3"/>
       <c r="L78" s="2" t="s">
@@ -5151,31 +5268,31 @@
         <v>25</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="I79" s="3" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="K79" s="3"/>
       <c r="L79" s="2" t="s">
@@ -5187,6 +5304,19 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="M14:M79">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M14:M79" xr:uid="{777D6F40-1F16-426E-B448-710C09E620C9}">
+      <formula1>"Pass,Fail"</formula1>
+    </dataValidation>
+  </dataValidations>
   <hyperlinks>
     <hyperlink ref="B5" r:id="rId1" xr:uid="{A9C43836-539D-4081-8B35-8FEAFF66F00B}"/>
     <hyperlink ref="O14" r:id="rId2" xr:uid="{6E2448A7-3E3A-4EC7-9A26-9D691343DC32}"/>
@@ -5202,11 +5332,18 @@
     <hyperlink ref="O24" r:id="rId12" xr:uid="{2B998C3F-3E9D-4783-BF1E-B571D6980D52}"/>
     <hyperlink ref="O25" r:id="rId13" xr:uid="{A9F91156-7544-416B-BABA-57F820D7A096}"/>
     <hyperlink ref="O26" r:id="rId14" xr:uid="{3F9B958A-D6BB-42DD-A59A-8097230A06A4}"/>
+    <hyperlink ref="O27" r:id="rId15" xr:uid="{8AE54B3E-1CA2-4844-AD7D-AFD16EA6285B}"/>
+    <hyperlink ref="O28" r:id="rId16" xr:uid="{9DD3537F-242A-4EBF-BF78-68E1BFE385F6}"/>
+    <hyperlink ref="O29" r:id="rId17" xr:uid="{36EFE8EA-35A0-4CE8-9456-E694218FCA69}"/>
+    <hyperlink ref="O30" r:id="rId18" xr:uid="{20A9B1DB-DD75-487D-BD20-F2923B38F0D1}"/>
+    <hyperlink ref="O31" r:id="rId19" xr:uid="{0C0E9B5A-03CD-4F4E-8111-FE345AC377B1}"/>
+    <hyperlink ref="O32" r:id="rId20" xr:uid="{2A9958E2-5BD8-40AB-BFF1-3A59063C7A20}"/>
+    <hyperlink ref="O33" r:id="rId21" xr:uid="{B86C8C83-7A78-48F6-92CF-AA1F7D8D618D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId15"/>
-    <tablePart r:id="rId16"/>
+    <tablePart r:id="rId22"/>
+    <tablePart r:id="rId23"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>